<commit_message>
Updated logger and updsend
</commit_message>
<xml_diff>
--- a/Docs/BoatPerformanceLoggerBOM.xlsx
+++ b/Docs/BoatPerformanceLoggerBOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jespe\Documents\PlatformIO\Projects\BoatPerformanceLogger\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6102CA40-63B4-4602-906A-1E3E9B27F91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{039E18A9-7CB3-4C3F-A637-1DD84C205517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D7228C54-2EA5-4596-A6B2-9B57DAF4E7B7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{D7228C54-2EA5-4596-A6B2-9B57DAF4E7B7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="37">
   <si>
     <t>BoatPerformanceLogger - PlutoidEngineering</t>
   </si>
@@ -132,6 +132,24 @@
   </si>
   <si>
     <t>HDMI Skärm</t>
+  </si>
+  <si>
+    <t>Inköpslista - SensorESP</t>
+  </si>
+  <si>
+    <t>ESP32-S3</t>
+  </si>
+  <si>
+    <t>https://www.amazon.se/dp/B0FZGSR8NS</t>
+  </si>
+  <si>
+    <t>Passiv kylning till RPI</t>
+  </si>
+  <si>
+    <t>Behöver hitta en lämplig modell</t>
+  </si>
+  <si>
+    <t>Oklart</t>
   </si>
 </sst>
 </file>
@@ -202,16 +220,18 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -548,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E57F0C6E-83BB-40B4-9912-9C1BD6C95FB8}">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.28515625" bestFit="1" customWidth="1"/>
@@ -562,26 +582,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="8">
+        <f xml:space="preserve"> SUM(G3:G100)</f>
+        <v>565.5924</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="8">
+        <f xml:space="preserve"> SUM(I3:I100)</f>
+        <v>819.04</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
       <c r="F3" s="2" t="s">
         <v>21</v>
       </c>
@@ -635,7 +665,7 @@
         <f xml:space="preserve"> B5 * C5</f>
         <v>41.1</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F5" t="s">
@@ -656,7 +686,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <f t="shared" ref="D6:D11" si="0" xml:space="preserve"> B6 * C6</f>
+        <f t="shared" ref="D6:D10" si="0" xml:space="preserve"> B6 * C6</f>
         <v>0</v>
       </c>
       <c r="F6" t="s">
@@ -678,7 +708,7 @@
         <f t="shared" si="0"/>
         <v>28.82</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>11</v>
       </c>
       <c r="F7" t="s">
@@ -741,7 +771,7 @@
         <f t="shared" si="0"/>
         <v>87.68</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>20</v>
       </c>
       <c r="F10" t="s">
@@ -754,7 +784,7 @@
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C11" s="4"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="6"/>
+      <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C12" s="4"/>
@@ -769,13 +799,13 @@
       <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:9" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
       <c r="F15" s="2" t="s">
         <v>21</v>
       </c>
@@ -828,7 +858,7 @@
         <f t="shared" ref="D17:D31" si="2" xml:space="preserve"> B17 * C17</f>
         <v>99</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="5" t="s">
         <v>24</v>
       </c>
       <c r="F17" t="s">
@@ -863,10 +893,19 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>34</v>
+      </c>
       <c r="C19" s="4"/>
       <c r="D19" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
+      </c>
+      <c r="F19" t="s">
+        <v>35</v>
+      </c>
+      <c r="G19" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -953,11 +992,181 @@
         <v>0</v>
       </c>
     </row>
+    <row r="33" spans="1:9" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A33" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" s="3">
+        <f xml:space="preserve"> SUM(C35:C42)</f>
+        <v>98</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I33" s="3">
+        <f xml:space="preserve"> SUM(D35:D42)</f>
+        <v>196</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34" t="s">
+        <v>3</v>
+      </c>
+      <c r="C34" t="s">
+        <v>2</v>
+      </c>
+      <c r="D34" t="s">
+        <v>4</v>
+      </c>
+      <c r="E34" t="s">
+        <v>5</v>
+      </c>
+      <c r="F34" t="s">
+        <v>7</v>
+      </c>
+      <c r="G34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" s="4">
+        <f xml:space="preserve"> 196 / 2</f>
+        <v>98</v>
+      </c>
+      <c r="D35" s="1">
+        <f t="shared" ref="D35:D49" si="3" xml:space="preserve"> B35 * C35</f>
+        <v>196</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G35" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" s="4"/>
+      <c r="D36" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C37" s="4"/>
+      <c r="D37" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C38" s="4"/>
+      <c r="D38" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C39" s="4"/>
+      <c r="D39" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C40" s="4"/>
+      <c r="D40" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C41" s="4"/>
+      <c r="D41" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C42" s="4"/>
+      <c r="D42" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C43" s="4"/>
+      <c r="D43" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C44" s="4"/>
+      <c r="D44" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C45" s="4"/>
+      <c r="D45" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C46" s="4"/>
+      <c r="D46" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C47" s="4"/>
+      <c r="D47" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C48" s="4"/>
+      <c r="D48" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C49" s="4"/>
+      <c r="D49" s="1">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E17" r:id="rId1" xr:uid="{F4341D42-1AAE-45D4-B49B-10212614FE39}"/>

</xml_diff>